<commit_message>
fdsafdsafadsfdsafadsfdasfdsafdasferu9t8vh54yherdzjfh gqer7iujeldu sufxfhxjfh cdufujsdif hrvuadfhduxj
</commit_message>
<xml_diff>
--- a/Experimenten.xlsx
+++ b/Experimenten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stichtingfontys-my.sharepoint.com/personal/582755_student_fontys_nl/Documents/Leerjaar 2/Periode 1/Operations Research 5/OR5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="11_E1A8E876E44D7F44EB205E5B54E1B21826485FC6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AFB4758-D5B2-4F1C-B3FC-FDE4D9A4E4C6}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="11_E1A8E876E44D7F44EB205E5B54E1B21826485FC6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39CB30F0-1C33-45B3-9033-89D67EB5BB63}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,20 @@
     <sheet name="temp" sheetId="4" r:id="rId4"/>
     <sheet name="random_seed" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>